<commit_message>
Updated BIH_grids_kan10 model - 2026-08-27 13:24
</commit_message>
<xml_diff>
--- a/VerveStacks_BIH_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BIH_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BIH_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE45D629-1BE2-4C5A-B9E5-9A2AD8B6BA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45792F3E-FF80-4CC1-8344-2F0B7B8B6CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4357" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4372" uniqueCount="548">
   <si>
     <t>Unit</t>
   </si>
@@ -1282,15 +1282,15 @@
     <t>p_Mostar_BIH</t>
   </si>
   <si>
-    <t>p_Vogosca_BIH</t>
-  </si>
-  <si>
     <t>p_Bijeljina_BIH</t>
   </si>
   <si>
     <t>p_Trebinje_BIH</t>
   </si>
   <si>
+    <t>p_Travnik_BIH</t>
+  </si>
+  <si>
     <t>p_Doboj_BIH</t>
   </si>
   <si>
@@ -1300,12 +1300,15 @@
     <t>p_Bratunac_BIH</t>
   </si>
   <si>
-    <t>p_Zenica_BIH</t>
-  </si>
-  <si>
     <t>p_SirokiBrijeg_BIH</t>
   </si>
   <si>
+    <t>p_Orasje_BIH</t>
+  </si>
+  <si>
+    <t>p_Sarajevo_BIH</t>
+  </si>
+  <si>
     <t>s_ogci11364_BIH</t>
   </si>
   <si>
@@ -1390,33 +1393,39 @@
     <t>Herzegovina-Neretva</t>
   </si>
   <si>
+    <t>Bijeljina</t>
+  </si>
+  <si>
+    <t>Trebinje</t>
+  </si>
+  <si>
+    <t>Central Bosnia</t>
+  </si>
+  <si>
+    <t>Tuzla</t>
+  </si>
+  <si>
+    <t>Serbia - jug</t>
+  </si>
+  <si>
+    <t>Hrvatska</t>
+  </si>
+  <si>
+    <t>Zenica-Doboj</t>
+  </si>
+  <si>
+    <t>West Bosnia</t>
+  </si>
+  <si>
+    <t>West Herzegovina</t>
+  </si>
+  <si>
+    <t>Una-Sana</t>
+  </si>
+  <si>
     <t>Sarajevo</t>
   </si>
   <si>
-    <t>Bijeljina</t>
-  </si>
-  <si>
-    <t>Trebinje</t>
-  </si>
-  <si>
-    <t>Tuzla</t>
-  </si>
-  <si>
-    <t>Serbia - jug</t>
-  </si>
-  <si>
-    <t>Zenica-Doboj</t>
-  </si>
-  <si>
-    <t>West Bosnia</t>
-  </si>
-  <si>
-    <t>West Herzegovina</t>
-  </si>
-  <si>
-    <t>Una-Sana</t>
-  </si>
-  <si>
     <t>Sarajevo-romanija</t>
   </si>
   <si>
@@ -1435,15 +1444,15 @@
     <t>e_Mostar_BIH</t>
   </si>
   <si>
-    <t>e_Vogosca_BIH</t>
-  </si>
-  <si>
     <t>e_Bijeljina_BIH</t>
   </si>
   <si>
     <t>e_Trebinje_BIH</t>
   </si>
   <si>
+    <t>e_Travnik_BIH</t>
+  </si>
+  <si>
     <t>e_Doboj_BIH</t>
   </si>
   <si>
@@ -1453,12 +1462,15 @@
     <t>e_Bratunac_BIH</t>
   </si>
   <si>
-    <t>e_Zenica_BIH</t>
-  </si>
-  <si>
     <t>e_SirokiBrijeg_BIH</t>
   </si>
   <si>
+    <t>e_Orasje_BIH</t>
+  </si>
+  <si>
+    <t>e_Sarajevo_BIH</t>
+  </si>
+  <si>
     <t>elc_spv_BIH_001</t>
   </si>
   <si>
@@ -1537,15 +1549,15 @@
     <t>co2_Mostar_BIH</t>
   </si>
   <si>
-    <t>co2_Vogosca_BIH</t>
-  </si>
-  <si>
     <t>co2_Bijeljina_BIH</t>
   </si>
   <si>
     <t>co2_Trebinje_BIH</t>
   </si>
   <si>
+    <t>co2_Travnik_BIH</t>
+  </si>
+  <si>
     <t>co2_Doboj_BIH</t>
   </si>
   <si>
@@ -1555,12 +1567,15 @@
     <t>co2_Bratunac_BIH</t>
   </si>
   <si>
-    <t>co2_Zenica_BIH</t>
-  </si>
-  <si>
     <t>co2_SirokiBrijeg_BIH</t>
   </si>
   <si>
+    <t>co2_Orasje_BIH</t>
+  </si>
+  <si>
+    <t>co2_Sarajevo_BIH</t>
+  </si>
+  <si>
     <t>co2s_ogci11364_BIH</t>
   </si>
   <si>
@@ -1579,15 +1594,15 @@
     <t>BIH-e_Mostar_BIH</t>
   </si>
   <si>
-    <t>BIH-e_Vogosca_BIH</t>
-  </si>
-  <si>
     <t>BIH-e_Bijeljina_BIH</t>
   </si>
   <si>
     <t>BIH-e_Trebinje_BIH</t>
   </si>
   <si>
+    <t>BIH-e_Travnik_BIH</t>
+  </si>
+  <si>
     <t>BIH-e_Doboj_BIH</t>
   </si>
   <si>
@@ -1597,12 +1612,15 @@
     <t>BIH-e_Bratunac_BIH</t>
   </si>
   <si>
-    <t>BIH-e_Zenica_BIH</t>
-  </si>
-  <si>
     <t>BIH-e_SirokiBrijeg_BIH</t>
   </si>
   <si>
+    <t>BIH-e_Orasje_BIH</t>
+  </si>
+  <si>
+    <t>BIH-e_Sarajevo_BIH</t>
+  </si>
+  <si>
     <t>BIH-elc_spv_BIH_001</t>
   </si>
   <si>
@@ -1681,15 +1699,15 @@
     <t>BIH-co2_Mostar_BIH</t>
   </si>
   <si>
-    <t>BIH-co2_Vogosca_BIH</t>
-  </si>
-  <si>
     <t>BIH-co2_Bijeljina_BIH</t>
   </si>
   <si>
     <t>BIH-co2_Trebinje_BIH</t>
   </si>
   <si>
+    <t>BIH-co2_Travnik_BIH</t>
+  </si>
+  <si>
     <t>BIH-co2_Doboj_BIH</t>
   </si>
   <si>
@@ -1699,10 +1717,13 @@
     <t>BIH-co2_Bratunac_BIH</t>
   </si>
   <si>
-    <t>BIH-co2_Zenica_BIH</t>
-  </si>
-  <si>
     <t>BIH-co2_SirokiBrijeg_BIH</t>
+  </si>
+  <si>
+    <t>BIH-co2_Orasje_BIH</t>
+  </si>
+  <si>
+    <t>BIH-co2_Sarajevo_BIH</t>
   </si>
   <si>
     <t>BIH-co2s_ogci11364_BIH</t>
@@ -2634,8 +2655,8 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55280901-1451-4371-936A-B0AE1D7C0B94}">
-  <dimension ref="B9:L55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{015D4376-8544-4608-82BF-DA86BC1A2E54}">
+  <dimension ref="B9:L57"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:12">
@@ -2692,19 +2713,19 @@
         <v>397</v>
       </c>
       <c r="G11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J11" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="L11" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="12" spans="2:12">
@@ -2721,19 +2742,19 @@
         <v>398</v>
       </c>
       <c r="G12" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H12" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K12" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="L12" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
     <row r="13" spans="2:12">
@@ -2750,19 +2771,19 @@
         <v>399</v>
       </c>
       <c r="G13" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H13" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J13" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K13" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="L13" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="14" spans="2:12">
@@ -2779,19 +2800,19 @@
         <v>400</v>
       </c>
       <c r="G14" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H14" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J14" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K14" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="L14" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="15" spans="2:12">
@@ -2808,19 +2829,19 @@
         <v>401</v>
       </c>
       <c r="G15" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K15" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="L15" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="16" spans="2:12">
@@ -2837,19 +2858,19 @@
         <v>402</v>
       </c>
       <c r="G16" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H16" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J16" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K16" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="L16" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="17" spans="2:12">
@@ -2866,19 +2887,19 @@
         <v>403</v>
       </c>
       <c r="G17" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H17" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J17" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K17" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="L17" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="2:12">
@@ -2895,19 +2916,19 @@
         <v>404</v>
       </c>
       <c r="G18" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H18" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J18" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K18" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="L18" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="19" spans="2:12">
@@ -2924,19 +2945,19 @@
         <v>405</v>
       </c>
       <c r="G19" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H19" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="J19" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K19" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="L19" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="20" spans="2:12">
@@ -2953,19 +2974,19 @@
         <v>406</v>
       </c>
       <c r="G20" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H20" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="J20" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K20" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="L20" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
     </row>
     <row r="21" spans="2:12">
@@ -2979,22 +3000,22 @@
         <v>407</v>
       </c>
       <c r="F21" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G21" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H21" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J21" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K21" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="L21" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="22" spans="2:12">
@@ -3011,19 +3032,19 @@
         <v>409</v>
       </c>
       <c r="G22" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H22" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="J22" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K22" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="L22" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="23" spans="2:12">
@@ -3040,19 +3061,19 @@
         <v>410</v>
       </c>
       <c r="G23" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H23" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="J23" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K23" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="L23" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
     <row r="24" spans="2:12">
@@ -3069,19 +3090,19 @@
         <v>411</v>
       </c>
       <c r="G24" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H24" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="J24" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K24" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="L24" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="25" spans="2:12">
@@ -3098,19 +3119,19 @@
         <v>412</v>
       </c>
       <c r="G25" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H25" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="J25" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K25" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="L25" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
     </row>
     <row r="26" spans="2:12">
@@ -3127,19 +3148,19 @@
         <v>413</v>
       </c>
       <c r="G26" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H26" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="J26" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K26" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="L26" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="27" spans="2:12">
@@ -3156,19 +3177,19 @@
         <v>414</v>
       </c>
       <c r="G27" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H27" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J27" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K27" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="L27" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="28" spans="2:12">
@@ -3185,19 +3206,19 @@
         <v>415</v>
       </c>
       <c r="G28" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H28" t="s">
-        <v>433</v>
+        <v>445</v>
       </c>
       <c r="J28" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K28" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="L28" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="29" spans="2:12">
@@ -3214,19 +3235,19 @@
         <v>416</v>
       </c>
       <c r="G29" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H29" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="J29" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K29" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="L29" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="30" spans="2:12">
@@ -3243,19 +3264,19 @@
         <v>417</v>
       </c>
       <c r="G30" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H30" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="J30" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K30" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="L30" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="31" spans="2:12">
@@ -3272,19 +3293,19 @@
         <v>418</v>
       </c>
       <c r="G31" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H31" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="J31" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K31" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="L31" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="32" spans="2:12">
@@ -3301,19 +3322,19 @@
         <v>419</v>
       </c>
       <c r="G32" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H32" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="J32" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K32" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="L32" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="33" spans="2:12">
@@ -3330,19 +3351,19 @@
         <v>420</v>
       </c>
       <c r="G33" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H33" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="J33" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K33" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="L33" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="34" spans="2:12">
@@ -3359,19 +3380,19 @@
         <v>421</v>
       </c>
       <c r="G34" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H34" t="s">
-        <v>445</v>
+        <v>434</v>
       </c>
       <c r="J34" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K34" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="L34" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="35" spans="2:12">
@@ -3388,19 +3409,19 @@
         <v>422</v>
       </c>
       <c r="G35" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H35" t="s">
-        <v>437</v>
+        <v>448</v>
       </c>
       <c r="J35" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K35" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="L35" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="36" spans="2:12">
@@ -3417,19 +3438,19 @@
         <v>423</v>
       </c>
       <c r="G36" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H36" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="J36" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K36" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="L36" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="37" spans="2:12">
@@ -3446,19 +3467,19 @@
         <v>424</v>
       </c>
       <c r="G37" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H37" t="s">
-        <v>434</v>
+        <v>449</v>
       </c>
       <c r="J37" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K37" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="L37" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="38" spans="2:12">
@@ -3475,19 +3496,19 @@
         <v>425</v>
       </c>
       <c r="G38" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H38" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J38" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K38" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="L38" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="39" spans="2:12">
@@ -3504,19 +3525,19 @@
         <v>426</v>
       </c>
       <c r="G39" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H39" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="J39" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K39" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="L39" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="40" spans="2:12">
@@ -3533,19 +3554,19 @@
         <v>427</v>
       </c>
       <c r="G40" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H40" t="s">
-        <v>436</v>
+        <v>448</v>
       </c>
       <c r="J40" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K40" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="L40" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
     </row>
     <row r="41" spans="2:12">
@@ -3562,19 +3583,19 @@
         <v>428</v>
       </c>
       <c r="G41" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H41" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="J41" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K41" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="L41" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="42" spans="2:12">
@@ -3591,19 +3612,19 @@
         <v>429</v>
       </c>
       <c r="G42" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H42" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J42" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K42" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="L42" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
     </row>
     <row r="43" spans="2:12">
@@ -3620,19 +3641,19 @@
         <v>430</v>
       </c>
       <c r="G43" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H43" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="J43" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K43" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="L43" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="44" spans="2:12">
@@ -3649,19 +3670,19 @@
         <v>431</v>
       </c>
       <c r="G44" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H44" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="J44" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K44" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="L44" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="45" spans="2:12">
@@ -3675,132 +3696,172 @@
         <v>431</v>
       </c>
       <c r="F45" t="s">
-        <v>407</v>
+        <v>432</v>
       </c>
       <c r="G45" t="s">
+        <v>433</v>
+      </c>
+      <c r="H45" t="s">
+        <v>443</v>
+      </c>
+      <c r="J45" t="s">
+        <v>450</v>
+      </c>
+      <c r="K45" t="s">
+        <v>485</v>
+      </c>
+      <c r="L45" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="46" spans="2:12">
+      <c r="B46" t="s">
+        <v>396</v>
+      </c>
+      <c r="C46" t="s">
         <v>432</v>
       </c>
-      <c r="H45" t="s">
-        <v>440</v>
-      </c>
-      <c r="J45" t="s">
-        <v>447</v>
-      </c>
-      <c r="K45" t="s">
-        <v>482</v>
-      </c>
-      <c r="L45" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12">
+      <c r="D46" t="s">
+        <v>432</v>
+      </c>
+      <c r="F46" t="s">
+        <v>408</v>
+      </c>
+      <c r="G46" t="s">
+        <v>433</v>
+      </c>
+      <c r="H46" t="s">
+        <v>442</v>
+      </c>
       <c r="J46" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K46" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="L46" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
     </row>
     <row r="47" spans="2:12">
       <c r="J47" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K47" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="L47" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="48" spans="2:12">
       <c r="J48" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K48" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="L48" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="49" spans="10:12">
       <c r="J49" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K49" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="L49" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="50" spans="10:12">
       <c r="J50" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K50" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="L50" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="51" spans="10:12">
       <c r="J51" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K51" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="L51" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="52" spans="10:12">
       <c r="J52" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K52" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="L52" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="53" spans="10:12">
       <c r="J53" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K53" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="L53" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="54" spans="10:12">
       <c r="J54" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K54" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="L54" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="55" spans="10:12">
       <c r="J55" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K55" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="L55" t="s">
-        <v>492</v>
+        <v>495</v>
+      </c>
+    </row>
+    <row r="56" spans="10:12">
+      <c r="J56" t="s">
+        <v>450</v>
+      </c>
+      <c r="K56" t="s">
+        <v>496</v>
+      </c>
+      <c r="L56" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="57" spans="10:12">
+      <c r="J57" t="s">
+        <v>450</v>
+      </c>
+      <c r="K57" t="s">
+        <v>497</v>
+      </c>
+      <c r="L57" t="s">
+        <v>497</v>
       </c>
     </row>
   </sheetData>
@@ -20867,16 +20928,16 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FF0BC6-B93C-4656-9388-5D66C6AF2A0E}">
-  <dimension ref="B9:H55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A817E86F-269A-4437-A2FC-A9BC8C107AF3}">
+  <dimension ref="B9:H57"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="F9" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -20884,19 +20945,19 @@
         <v>389</v>
       </c>
       <c r="C10" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D10" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="F10" t="s">
         <v>389</v>
       </c>
       <c r="G10" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="H10" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
     </row>
     <row r="11" spans="2:8">
@@ -20910,7 +20971,7 @@
         <v>16.71876991179986</v>
       </c>
       <c r="F11" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="G11">
         <v>44.940994050093479</v>
@@ -20930,7 +20991,7 @@
         <v>17.76985819575496</v>
       </c>
       <c r="F12" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="G12">
         <v>43.303196306313311</v>
@@ -20944,19 +21005,19 @@
         <v>399</v>
       </c>
       <c r="C13">
-        <v>43.882748242161547</v>
+        <v>44.686458240245742</v>
       </c>
       <c r="D13">
-        <v>18.315516969695064</v>
+        <v>18.965914839988223</v>
       </c>
       <c r="F13" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="G13">
-        <v>43.882748242161547</v>
+        <v>44.686458240245742</v>
       </c>
       <c r="H13">
-        <v>18.315516969695064</v>
+        <v>18.965914839988223</v>
       </c>
     </row>
     <row r="14" spans="2:8">
@@ -20964,19 +21025,19 @@
         <v>400</v>
       </c>
       <c r="C14">
-        <v>44.686458240245742</v>
+        <v>42.677365387414312</v>
       </c>
       <c r="D14">
-        <v>18.965914839988223</v>
+        <v>18.333420931217962</v>
       </c>
       <c r="F14" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="G14">
-        <v>44.686458240245742</v>
+        <v>42.677365387414312</v>
       </c>
       <c r="H14">
-        <v>18.965914839988223</v>
+        <v>18.333420931217962</v>
       </c>
     </row>
     <row r="15" spans="2:8">
@@ -20984,19 +21045,19 @@
         <v>401</v>
       </c>
       <c r="C15">
-        <v>42.677365387414312</v>
+        <v>44.328637955431432</v>
       </c>
       <c r="D15">
-        <v>18.333420931217962</v>
+        <v>17.264451011210998</v>
       </c>
       <c r="F15" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="G15">
-        <v>42.677365387414312</v>
+        <v>44.328637955431432</v>
       </c>
       <c r="H15">
-        <v>18.333420931217962</v>
+        <v>17.264451011210998</v>
       </c>
     </row>
     <row r="16" spans="2:8">
@@ -21010,7 +21071,7 @@
         <v>18.435928500334398</v>
       </c>
       <c r="F16" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="G16">
         <v>44.90501355663578</v>
@@ -21024,19 +21085,19 @@
         <v>403</v>
       </c>
       <c r="C17">
-        <v>44.52231833808716</v>
+        <v>44.480477614181083</v>
       </c>
       <c r="D17">
-        <v>18.604885316340617</v>
+        <v>18.605783043969407</v>
       </c>
       <c r="F17" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="G17">
-        <v>44.52231833808716</v>
+        <v>44.480477614181083</v>
       </c>
       <c r="H17">
-        <v>18.604885316340617</v>
+        <v>18.605783043969407</v>
       </c>
     </row>
     <row r="18" spans="2:8">
@@ -21050,7 +21111,7 @@
         <v>19.499663482609684</v>
       </c>
       <c r="F18" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="G18">
         <v>43.953047577375791</v>
@@ -21064,19 +21125,19 @@
         <v>405</v>
       </c>
       <c r="C19">
-        <v>44.185989089314205</v>
+        <v>43.66018690912891</v>
       </c>
       <c r="D19">
-        <v>17.971015340419711</v>
+        <v>17.754869598202237</v>
       </c>
       <c r="F19" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="G19">
-        <v>44.185989089314205</v>
+        <v>43.66018690912891</v>
       </c>
       <c r="H19">
-        <v>17.971015340419711</v>
+        <v>17.754869598202237</v>
       </c>
     </row>
     <row r="20" spans="2:8">
@@ -21084,39 +21145,39 @@
         <v>406</v>
       </c>
       <c r="C20">
-        <v>43.66018690912891</v>
+        <v>45.287890541117157</v>
       </c>
       <c r="D20">
-        <v>17.754869598202237</v>
+        <v>18.42110605005314</v>
       </c>
       <c r="F20" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="G20">
-        <v>43.66018690912891</v>
+        <v>45.287890541117157</v>
       </c>
       <c r="H20">
-        <v>17.754869598202237</v>
+        <v>18.42110605005314</v>
       </c>
     </row>
     <row r="21" spans="2:8">
       <c r="B21" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C21">
-        <v>44.057613976118681</v>
+        <v>44.036557460947769</v>
       </c>
       <c r="D21">
-        <v>16.848113788793327</v>
+        <v>18.123210349406762</v>
       </c>
       <c r="F21" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="G21">
-        <v>44.057613976118681</v>
+        <v>44.036557460947769</v>
       </c>
       <c r="H21">
-        <v>16.848113788793327</v>
+        <v>18.123210349406762</v>
       </c>
     </row>
     <row r="22" spans="2:8">
@@ -21124,19 +21185,19 @@
         <v>409</v>
       </c>
       <c r="C22">
-        <v>43.465260169133238</v>
+        <v>44.057613976118681</v>
       </c>
       <c r="D22">
-        <v>17.378143623572235</v>
+        <v>16.848113788793327</v>
       </c>
       <c r="F22" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="G22">
-        <v>43.465260169133238</v>
+        <v>44.057613976118681</v>
       </c>
       <c r="H22">
-        <v>17.378143623572235</v>
+        <v>16.848113788793327</v>
       </c>
     </row>
     <row r="23" spans="2:8">
@@ -21144,19 +21205,19 @@
         <v>410</v>
       </c>
       <c r="C23">
-        <v>42.956173893431625</v>
+        <v>43.465260169133238</v>
       </c>
       <c r="D23">
-        <v>18.311731015800159</v>
+        <v>17.378143623572235</v>
       </c>
       <c r="F23" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="G23">
-        <v>42.956173893431625</v>
+        <v>43.465260169133238</v>
       </c>
       <c r="H23">
-        <v>18.311731015800159</v>
+        <v>17.378143623572235</v>
       </c>
     </row>
     <row r="24" spans="2:8">
@@ -21164,19 +21225,19 @@
         <v>411</v>
       </c>
       <c r="C24">
-        <v>43.87828927556837</v>
+        <v>42.956173893431625</v>
       </c>
       <c r="D24">
-        <v>17.444108263455796</v>
+        <v>18.311731015800159</v>
       </c>
       <c r="F24" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="G24">
-        <v>43.87828927556837</v>
+        <v>42.956173893431625</v>
       </c>
       <c r="H24">
-        <v>17.444108263455796</v>
+        <v>18.311731015800159</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -21184,19 +21245,19 @@
         <v>412</v>
       </c>
       <c r="C25">
-        <v>43.428769171441658</v>
+        <v>43.87828927556837</v>
       </c>
       <c r="D25">
-        <v>18.276658083463406</v>
+        <v>17.444108263455796</v>
       </c>
       <c r="F25" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="G25">
-        <v>43.428769171441658</v>
+        <v>43.87828927556837</v>
       </c>
       <c r="H25">
-        <v>18.276658083463406</v>
+        <v>17.444108263455796</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -21204,19 +21265,19 @@
         <v>413</v>
       </c>
       <c r="C26">
-        <v>45.002744611515183</v>
+        <v>43.428769171441658</v>
       </c>
       <c r="D26">
-        <v>15.978434643716612</v>
+        <v>18.276658083463406</v>
       </c>
       <c r="F26" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="G26">
-        <v>45.002744611515183</v>
+        <v>43.428769171441658</v>
       </c>
       <c r="H26">
-        <v>15.978434643716612</v>
+        <v>18.276658083463406</v>
       </c>
     </row>
     <row r="27" spans="2:8">
@@ -21224,19 +21285,19 @@
         <v>414</v>
       </c>
       <c r="C27">
-        <v>44.606501079376017</v>
+        <v>45.002744611515183</v>
       </c>
       <c r="D27">
-        <v>16.29623575978405</v>
+        <v>15.978434643716612</v>
       </c>
       <c r="F27" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="G27">
-        <v>44.606501079376017</v>
+        <v>45.002744611515183</v>
       </c>
       <c r="H27">
-        <v>16.29623575978405</v>
+        <v>15.978434643716612</v>
       </c>
     </row>
     <row r="28" spans="2:8">
@@ -21244,19 +21305,19 @@
         <v>415</v>
       </c>
       <c r="C28">
-        <v>44.609096263080872</v>
+        <v>44.606501079376017</v>
       </c>
       <c r="D28">
-        <v>16.942960342572068</v>
+        <v>16.29623575978405</v>
       </c>
       <c r="F28" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="G28">
-        <v>44.609096263080872</v>
+        <v>44.606501079376017</v>
       </c>
       <c r="H28">
-        <v>16.942960342572068</v>
+        <v>16.29623575978405</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -21264,19 +21325,19 @@
         <v>416</v>
       </c>
       <c r="C29">
-        <v>45.047603057243791</v>
+        <v>44.609096263080872</v>
       </c>
       <c r="D29">
-        <v>16.748007185771105</v>
+        <v>16.942960342572068</v>
       </c>
       <c r="F29" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="G29">
-        <v>45.047603057243791</v>
+        <v>44.609096263080872</v>
       </c>
       <c r="H29">
-        <v>16.748007185771105</v>
+        <v>16.942960342572068</v>
       </c>
     </row>
     <row r="30" spans="2:8">
@@ -21284,19 +21345,19 @@
         <v>417</v>
       </c>
       <c r="C30">
-        <v>43.893677292673466</v>
+        <v>45.047603057243791</v>
       </c>
       <c r="D30">
-        <v>18.295289706978242</v>
+        <v>16.748007185771105</v>
       </c>
       <c r="F30" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="G30">
-        <v>43.893677292673466</v>
+        <v>45.047603057243791</v>
       </c>
       <c r="H30">
-        <v>18.295289706978242</v>
+        <v>16.748007185771105</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -21304,19 +21365,19 @@
         <v>418</v>
       </c>
       <c r="C31">
-        <v>43.887694891985447</v>
+        <v>43.893677292673466</v>
       </c>
       <c r="D31">
-        <v>19.110860975704451</v>
+        <v>18.295289706978242</v>
       </c>
       <c r="F31" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="G31">
-        <v>43.887694891985447</v>
+        <v>43.893677292673466</v>
       </c>
       <c r="H31">
-        <v>19.110860975704451</v>
+        <v>18.295289706978242</v>
       </c>
     </row>
     <row r="32" spans="2:8">
@@ -21324,19 +21385,19 @@
         <v>419</v>
       </c>
       <c r="C32">
-        <v>44.55016652983371</v>
+        <v>43.887694891985447</v>
       </c>
       <c r="D32">
-        <v>18.816376843269349</v>
+        <v>19.110860975704451</v>
       </c>
       <c r="F32" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="G32">
-        <v>44.55016652983371</v>
+        <v>43.887694891985447</v>
       </c>
       <c r="H32">
-        <v>18.816376843269349</v>
+        <v>19.110860975704451</v>
       </c>
     </row>
     <row r="33" spans="2:8">
@@ -21344,19 +21405,19 @@
         <v>420</v>
       </c>
       <c r="C33">
-        <v>44.618887511604576</v>
+        <v>44.55016652983371</v>
       </c>
       <c r="D33">
-        <v>17.765851307070299</v>
+        <v>18.816376843269349</v>
       </c>
       <c r="F33" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="G33">
-        <v>44.618887511604576</v>
+        <v>44.55016652983371</v>
       </c>
       <c r="H33">
-        <v>17.765851307070299</v>
+        <v>18.816376843269349</v>
       </c>
     </row>
     <row r="34" spans="2:8">
@@ -21364,19 +21425,19 @@
         <v>421</v>
       </c>
       <c r="C34">
-        <v>44.925715954776898</v>
+        <v>44.618887511604576</v>
       </c>
       <c r="D34">
-        <v>18.005228691426183</v>
+        <v>17.765851307070299</v>
       </c>
       <c r="F34" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="G34">
-        <v>44.925715954776898</v>
+        <v>44.618887511604576</v>
       </c>
       <c r="H34">
-        <v>18.005228691426183</v>
+        <v>17.765851307070299</v>
       </c>
     </row>
     <row r="35" spans="2:8">
@@ -21384,19 +21445,19 @@
         <v>422</v>
       </c>
       <c r="C35">
-        <v>42.953405544278802</v>
+        <v>44.925715954776898</v>
       </c>
       <c r="D35">
-        <v>18.32197152564548</v>
+        <v>18.005228691426183</v>
       </c>
       <c r="F35" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="G35">
-        <v>42.953405544278802</v>
+        <v>44.925715954776898</v>
       </c>
       <c r="H35">
-        <v>18.32197152564548</v>
+        <v>18.005228691426183</v>
       </c>
     </row>
     <row r="36" spans="2:8">
@@ -21404,19 +21465,19 @@
         <v>423</v>
       </c>
       <c r="C36">
-        <v>43.127075227327843</v>
+        <v>42.953405544278802</v>
       </c>
       <c r="D36">
-        <v>18.627262293368485</v>
+        <v>18.32197152564548</v>
       </c>
       <c r="F36" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="G36">
-        <v>43.127075227327843</v>
+        <v>42.953405544278802</v>
       </c>
       <c r="H36">
-        <v>18.627262293368485</v>
+        <v>18.32197152564548</v>
       </c>
     </row>
     <row r="37" spans="2:8">
@@ -21424,19 +21485,19 @@
         <v>424</v>
       </c>
       <c r="C37">
-        <v>42.948063383468678</v>
+        <v>43.127075227327843</v>
       </c>
       <c r="D37">
-        <v>18.016680757922487</v>
+        <v>18.627262293368485</v>
       </c>
       <c r="F37" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="G37">
-        <v>42.948063383468678</v>
+        <v>43.127075227327843</v>
       </c>
       <c r="H37">
-        <v>18.016680757922487</v>
+        <v>18.627262293368485</v>
       </c>
     </row>
     <row r="38" spans="2:8">
@@ -21444,19 +21505,19 @@
         <v>425</v>
       </c>
       <c r="C38">
-        <v>43.127075227327843</v>
+        <v>42.948063383468678</v>
       </c>
       <c r="D38">
-        <v>17.711389990199486</v>
+        <v>18.016680757922487</v>
       </c>
       <c r="F38" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="G38">
-        <v>43.127075227327843</v>
+        <v>42.948063383468678</v>
       </c>
       <c r="H38">
-        <v>17.711389990199486</v>
+        <v>18.016680757922487</v>
       </c>
     </row>
     <row r="39" spans="2:8">
@@ -21464,19 +21525,19 @@
         <v>426</v>
       </c>
       <c r="C39">
-        <v>44.925715954776905</v>
+        <v>43.127075227327843</v>
       </c>
       <c r="D39">
-        <v>18.627262293368485</v>
+        <v>17.711389990199486</v>
       </c>
       <c r="F39" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="G39">
-        <v>44.925715954776905</v>
+        <v>43.127075227327843</v>
       </c>
       <c r="H39">
-        <v>18.627262293368485</v>
+        <v>17.711389990199486</v>
       </c>
     </row>
     <row r="40" spans="2:8">
@@ -21484,19 +21545,19 @@
         <v>427</v>
       </c>
       <c r="C40">
-        <v>44.700885863845777</v>
+        <v>44.925715954776905</v>
       </c>
       <c r="D40">
-        <v>19.23784382881448</v>
+        <v>18.627262293368485</v>
       </c>
       <c r="F40" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="G40">
-        <v>44.700885863845777</v>
+        <v>44.925715954776905</v>
       </c>
       <c r="H40">
-        <v>19.23784382881448</v>
+        <v>18.627262293368485</v>
       </c>
     </row>
     <row r="41" spans="2:8">
@@ -21504,19 +21565,19 @@
         <v>428</v>
       </c>
       <c r="C41">
-        <v>44.476055772914641</v>
+        <v>44.700885863845777</v>
       </c>
       <c r="D41">
-        <v>16.184936151584491</v>
+        <v>19.23784382881448</v>
       </c>
       <c r="F41" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="G41">
-        <v>44.476055772914641</v>
+        <v>44.700885863845777</v>
       </c>
       <c r="H41">
-        <v>16.184936151584491</v>
+        <v>19.23784382881448</v>
       </c>
     </row>
     <row r="42" spans="2:8">
@@ -21524,16 +21585,16 @@
         <v>429</v>
       </c>
       <c r="C42">
-        <v>44.700885863845777</v>
+        <v>44.476055772914641</v>
       </c>
       <c r="D42">
         <v>16.184936151584491</v>
       </c>
       <c r="F42" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="G42">
-        <v>44.700885863845777</v>
+        <v>44.476055772914641</v>
       </c>
       <c r="H42">
         <v>16.184936151584491</v>
@@ -21544,19 +21605,19 @@
         <v>430</v>
       </c>
       <c r="C43">
-        <v>43.851912946765857</v>
+        <v>44.700885863845777</v>
       </c>
       <c r="D43">
-        <v>17.054788284677237</v>
+        <v>16.184936151584491</v>
       </c>
       <c r="F43" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="G43">
-        <v>43.851912946765857</v>
+        <v>44.700885863845777</v>
       </c>
       <c r="H43">
-        <v>17.054788284677237</v>
+        <v>16.184936151584491</v>
       </c>
     </row>
     <row r="44" spans="2:8">
@@ -21564,66 +21625,75 @@
         <v>431</v>
       </c>
       <c r="C44">
-        <v>43.801565500121242</v>
+        <v>43.851912946765857</v>
       </c>
       <c r="D44">
-        <v>16.795517687030493</v>
+        <v>17.054788284677237</v>
       </c>
       <c r="F44" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="G44">
-        <v>43.801565500121242</v>
+        <v>43.851912946765857</v>
       </c>
       <c r="H44">
-        <v>16.795517687030493</v>
+        <v>17.054788284677237</v>
       </c>
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>407</v>
+        <v>432</v>
       </c>
       <c r="C45">
+        <v>43.801565500121242</v>
+      </c>
+      <c r="D45">
+        <v>16.795517687030493</v>
+      </c>
+      <c r="F45" t="s">
+        <v>535</v>
+      </c>
+      <c r="G45">
+        <v>43.801565500121242</v>
+      </c>
+      <c r="H45">
+        <v>16.795517687030493</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8">
+      <c r="B46" t="s">
+        <v>408</v>
+      </c>
+      <c r="C46">
         <v>44.051400000000001</v>
       </c>
-      <c r="D45">
+      <c r="D46">
         <v>18.103400000000001</v>
       </c>
-      <c r="F45" t="s">
-        <v>530</v>
-      </c>
-      <c r="G45">
+      <c r="F46" t="s">
+        <v>536</v>
+      </c>
+      <c r="G46">
         <v>44.940994050093479</v>
       </c>
-      <c r="H45">
+      <c r="H46">
         <v>16.71876991179986</v>
-      </c>
-    </row>
-    <row r="46" spans="2:8">
-      <c r="F46" t="s">
-        <v>531</v>
-      </c>
-      <c r="G46">
-        <v>43.303196306313311</v>
-      </c>
-      <c r="H46">
-        <v>17.76985819575496</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="F47" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="G47">
-        <v>43.882748242161547</v>
+        <v>43.303196306313311</v>
       </c>
       <c r="H47">
-        <v>18.315516969695064</v>
+        <v>17.76985819575496</v>
       </c>
     </row>
     <row r="48" spans="2:8">
       <c r="F48" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="G48">
         <v>44.686458240245742</v>
@@ -21634,7 +21704,7 @@
     </row>
     <row r="49" spans="6:8">
       <c r="F49" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="G49">
         <v>42.677365387414312</v>
@@ -21645,51 +21715,51 @@
     </row>
     <row r="50" spans="6:8">
       <c r="F50" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="G50">
-        <v>44.90501355663578</v>
+        <v>44.328637955431432</v>
       </c>
       <c r="H50">
-        <v>18.435928500334398</v>
+        <v>17.264451011210998</v>
       </c>
     </row>
     <row r="51" spans="6:8">
       <c r="F51" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="G51">
-        <v>44.52231833808716</v>
+        <v>44.90501355663578</v>
       </c>
       <c r="H51">
-        <v>18.604885316340617</v>
+        <v>18.435928500334398</v>
       </c>
     </row>
     <row r="52" spans="6:8">
       <c r="F52" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="G52">
-        <v>43.953047577375791</v>
+        <v>44.480477614181083</v>
       </c>
       <c r="H52">
-        <v>19.499663482609684</v>
+        <v>18.605783043969407</v>
       </c>
     </row>
     <row r="53" spans="6:8">
       <c r="F53" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="G53">
-        <v>44.185989089314205</v>
+        <v>43.953047577375791</v>
       </c>
       <c r="H53">
-        <v>17.971015340419711</v>
+        <v>19.499663482609684</v>
       </c>
     </row>
     <row r="54" spans="6:8">
       <c r="F54" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="G54">
         <v>43.66018690912891</v>
@@ -21700,12 +21770,34 @@
     </row>
     <row r="55" spans="6:8">
       <c r="F55" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="G55">
+        <v>45.287890541117157</v>
+      </c>
+      <c r="H55">
+        <v>18.42110605005314</v>
+      </c>
+    </row>
+    <row r="56" spans="6:8">
+      <c r="F56" t="s">
+        <v>546</v>
+      </c>
+      <c r="G56">
+        <v>44.036557460947769</v>
+      </c>
+      <c r="H56">
+        <v>18.123210349406762</v>
+      </c>
+    </row>
+    <row r="57" spans="6:8">
+      <c r="F57" t="s">
+        <v>547</v>
+      </c>
+      <c r="G57">
         <v>44.051400000000001</v>
       </c>
-      <c r="H55">
+      <c r="H57">
         <v>18.103400000000001</v>
       </c>
     </row>

</xml_diff>